<commit_message>
Complete Birth validation engine and generic rule framework
</commit_message>
<xml_diff>
--- a/data/output/summaries/summary_report.xlsx
+++ b/data/output/summaries/summary_report.xlsx
@@ -460,7 +460,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 10:03:47</t>
+          <t>2026-07-11 12:21:23</t>
         </is>
       </c>
     </row>
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>136</v>
+        <v>671</v>
       </c>
     </row>
     <row r="5">
@@ -492,7 +492,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>67.15%</t>
+          <t>-62.08%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implemented complete Death dataset validation pipeline
</commit_message>
<xml_diff>
--- a/data/output/summaries/summary_report.xlsx
+++ b/data/output/summaries/summary_report.xlsx
@@ -460,7 +460,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 13:14:10</t>
+          <t>2026-07-11 21:33:26</t>
         </is>
       </c>
     </row>
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="4">
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>671</v>
+        <v>2222</v>
       </c>
     </row>
     <row r="5">
@@ -492,7 +492,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>-62.08%</t>
+          <t>-440.63%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 5: Added intelligent schema detection, placeholder handling, validation improvements, status rules and reporting refactor
</commit_message>
<xml_diff>
--- a/data/output/summaries/summary_report.xlsx
+++ b/data/output/summaries/summary_report.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,10 +433,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -459,7 +459,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>411</v>
+        <v>305</v>
       </c>
     </row>
     <row r="3">
@@ -469,7 +469,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4">
@@ -479,7 +479,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>177</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5">
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>56.93</v>
+        <v>82.3</v>
       </c>
     </row>
     <row r="6"/>
@@ -509,260 +509,60 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>id_number</t>
+          <t>registration_date</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>100</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>registration_date</t>
+          <t>mother_age</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>date_of_death</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>sex</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>age</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>2</v>
-      </c>
-    </row>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>age_unit</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>2</v>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Issues</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>place_of_death</t>
+          <t>registration_date</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>place_type</t>
+          <t>mother_age</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>residence</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>marital_status</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>cause_of_death</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>death_certification</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>entry_number</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Rule</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Issues</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>DateConsistencyRule</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>SexRule</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>AgeRule</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>AgeUnitRule</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>PlaceOfDeathRule</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>PlaceTypeRule</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>ResidenceRule</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>MaritalStatusRule</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>CauseOfDeathRule</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>CertificationRule</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>EntryNumberRule</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B36"/>
+  <autoFilter ref="A1:B16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor GUI into modular components and rebuild main window
</commit_message>
<xml_diff>
--- a/data/output/summaries/summary_report.xlsx
+++ b/data/output/summaries/summary_report.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,10 +433,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -479,7 +479,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>54</v>
+        <v>155</v>
       </c>
     </row>
     <row r="5">
@@ -489,80 +489,76 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>82.3</v>
-      </c>
-    </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+        <v>49.18</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Current Registrations</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Late Registrations</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Issues</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>registration_date</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B13" t="n">
         <v>53</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>mother_age</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Rule</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Issues</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>registration_date</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
           <t>mother_age</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B14" t="n">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B16"/>
+  <autoFilter ref="A1:B14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>